<commit_message>
Atualizando versão dos pacotes e realizando upgrade para .NET 9
</commit_message>
<xml_diff>
--- a/arquivos/REM22062023_BIKE.xlsx
+++ b/arquivos/REM22062023_BIKE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorios\GIT - Pessoal\File Management\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF5C372-FB0B-4C7C-A00B-5D2D56503848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CFF4B6-012F-4A9B-B4A4-EB02FACFBA4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="12">
   <si>
     <t>Jose</t>
   </si>
   <si>
-    <t>Fernando</t>
-  </si>
-  <si>
     <t>Bike</t>
   </si>
   <si>
@@ -49,6 +46,21 @@
   </si>
   <si>
     <t>IsNew</t>
+  </si>
+  <si>
+    <t>Luis</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>Pedro</t>
+  </si>
+  <si>
+    <t>Rafael</t>
+  </si>
+  <si>
+    <t>Lucas</t>
   </si>
 </sst>
 </file>
@@ -374,255 +386,255 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14" t="s">
         <v>0</v>
       </c>
       <c r="C14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" t="s">
         <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>